<commit_message>
Update project and confusion matrix
</commit_message>
<xml_diff>
--- a/datasets/01_raw_data_3000.xlsx
+++ b/datasets/01_raw_data_3000.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ADMIN\Desktop\HealthDiagnosisApp\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718266ED-581E-420D-8986-E875209A828D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02D0621-CCA0-4233-A054-03BBD13B689D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17160,7 +17160,7 @@
     <col min="2" max="2" width="4.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="84.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="55.6640625" customWidth="1"/>
     <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>

</xml_diff>